<commit_message>
Set the manuscript in the double-spaced Times letter layout.
Center the title, article type, and author, and keep the same KG-EWS results, tables, and figure.

Co-authored-by: hemasribabburu <hemasribabburu@gmail.com>
</commit_message>
<xml_diff>
--- a/DBA802_Hemasri_Babburu_Final_Assignment/DBA802_Assignment_Compliance_Checklist.xlsx
+++ b/DBA802_Hemasri_Babburu_Final_Assignment/DBA802_Assignment_Compliance_Checklist.xlsx
@@ -595,12 +595,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Reference list is compact so the short communication stays within 10 pages.</t>
+          <t>The file is 12 double-spaced letter pages. The journal short-communication cap is 10 pages.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>10 letter pages, one embedded figure, two tables.</t>
+          <t>12 letter pages, one figure, two tables. Times New Roman.</t>
         </is>
       </c>
     </row>

</xml_diff>